<commit_message>
fixed library to work with pdf
</commit_message>
<xml_diff>
--- a/Test Participant.xlsx
+++ b/Test Participant.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samueladesoga/projects/cert_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536592A8-551A-CB46-AA8A-5F65555999BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BCA4FE4-5C15-F44F-806C-32C6FE90F01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="14960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40" yWindow="4720" windowWidth="30240" windowHeight="14960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Email</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Seun</t>
   </si>
   <si>
-    <t>Temitope</t>
-  </si>
-  <si>
     <t>samueladesoga@gmail.com</t>
   </si>
   <si>
@@ -46,13 +43,25 @@
     <t>Adesoga</t>
   </si>
   <si>
-    <t>temitope@valuehut.co</t>
-  </si>
-  <si>
-    <t>Dada</t>
-  </si>
-  <si>
     <t>samuel@valuehut.co</t>
+  </si>
+  <si>
+    <t>ea@valuehut.co</t>
+  </si>
+  <si>
+    <t>Funke</t>
+  </si>
+  <si>
+    <t>Jolayemi</t>
+  </si>
+  <si>
+    <t>Chisom</t>
+  </si>
+  <si>
+    <t>Michael</t>
+  </si>
+  <si>
+    <t xml:space="preserve">michaelchisomfortune@gmail.com </t>
   </si>
 </sst>
 </file>
@@ -419,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53" customWidth="1"/>
@@ -439,13 +448,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -453,21 +462,32 @@
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>